<commit_message>
refer type from other field
</commit_message>
<xml_diff>
--- a/test/res/item.xlsx
+++ b/test/res/item.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10810"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\bite\Desktop\github\xlsx-exporter\test\res\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/codetypes/Desktop/Github/xlsx-exporter/test/res/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABFD7722-8747-4444-861D-0F5876A3A679}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF113DD3-916C-AD43-A82F-1A0D070E0E3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-37740" yWindow="435" windowWidth="33675" windowHeight="19725" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17700" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="define" sheetId="2" r:id="rId1"/>
@@ -112,7 +112,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="119">
   <si>
     <t>id</t>
   </si>
@@ -479,31 +479,37 @@
   <si>
     <t>BagType</t>
     <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>@value_type</t>
+  </si>
+  <si>
+    <t>--</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -537,13 +543,13 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -551,7 +557,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -746,7 +752,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="常规 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
   </cellStyles>
   <dxfs count="6">
@@ -1076,18 +1082,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H18"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="14.875" customWidth="1"/>
-    <col min="3" max="3" width="24.125" customWidth="1"/>
-    <col min="4" max="4" width="21.125" customWidth="1"/>
-    <col min="5" max="5" width="20.375" customWidth="1"/>
-    <col min="6" max="6" width="8.5" customWidth="1"/>
-    <col min="7" max="7" width="9.625" customWidth="1"/>
-    <col min="8" max="8" width="18.375" style="16" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.1640625" customWidth="1"/>
+    <col min="4" max="4" width="21.1640625" customWidth="1"/>
+    <col min="5" max="5" width="20.33203125" customWidth="1"/>
+    <col min="6" max="6" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.6640625" customWidth="1"/>
+    <col min="8" max="8" width="18.33203125" style="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8">
       <c r="A1" s="29" t="s">
         <v>110</v>
       </c>
@@ -1099,7 +1105,7 @@
       <c r="G1" s="30"/>
       <c r="H1" s="30"/>
     </row>
-    <row r="2" spans="1:8" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" ht="16">
       <c r="A2" s="7" t="s">
         <v>0</v>
       </c>
@@ -1125,7 +1131,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" ht="16">
       <c r="A3" s="7" t="s">
         <v>63</v>
       </c>
@@ -1142,7 +1148,7 @@
         <v>64</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>12</v>
+        <v>117</v>
       </c>
       <c r="G3" s="8" t="s">
         <v>12</v>
@@ -1151,7 +1157,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" ht="16">
       <c r="A4" s="7" t="s">
         <v>15</v>
       </c>
@@ -1163,7 +1169,7 @@
       <c r="G4" s="8"/>
       <c r="H4" s="9"/>
     </row>
-    <row r="5" spans="1:8" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" ht="16">
       <c r="A5" s="7" t="s">
         <v>17</v>
       </c>
@@ -1189,7 +1195,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" ht="16">
       <c r="A6" s="7" t="s">
         <v>18</v>
       </c>
@@ -1205,7 +1211,7 @@
       <c r="G6" s="8"/>
       <c r="H6" s="9"/>
     </row>
-    <row r="7" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="16">
       <c r="A7" s="1" t="s">
         <v>65</v>
       </c>
@@ -1225,7 +1231,7 @@
       </c>
       <c r="H7" s="15"/>
     </row>
-    <row r="8" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" ht="16">
       <c r="A8" s="1" t="s">
         <v>65</v>
       </c>
@@ -1251,7 +1257,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" ht="16">
       <c r="A9" s="1" t="s">
         <v>65</v>
       </c>
@@ -1273,7 +1279,7 @@
       </c>
       <c r="H9" s="18"/>
     </row>
-    <row r="10" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" ht="16">
       <c r="A10" s="1" t="s">
         <v>65</v>
       </c>
@@ -1295,7 +1301,7 @@
       </c>
       <c r="H10" s="7"/>
     </row>
-    <row r="11" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" ht="16">
       <c r="A11" s="1" t="s">
         <v>65</v>
       </c>
@@ -1317,7 +1323,7 @@
       </c>
       <c r="H11" s="7"/>
     </row>
-    <row r="12" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" ht="16">
       <c r="A12" s="1" t="s">
         <v>65</v>
       </c>
@@ -1343,7 +1349,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" ht="16">
       <c r="A13" s="1" t="s">
         <v>65</v>
       </c>
@@ -1367,7 +1373,7 @@
       </c>
       <c r="H13" s="7"/>
     </row>
-    <row r="14" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" ht="16">
       <c r="A14" s="1" t="s">
         <v>65</v>
       </c>
@@ -1391,7 +1397,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" ht="16">
       <c r="A15" s="1" t="s">
         <v>65</v>
       </c>
@@ -1413,7 +1419,7 @@
       </c>
       <c r="H15" s="19"/>
     </row>
-    <row r="16" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" ht="16">
       <c r="A16" s="1" t="s">
         <v>65</v>
       </c>
@@ -1435,7 +1441,7 @@
       </c>
       <c r="H16" s="19"/>
     </row>
-    <row r="17" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" ht="16">
       <c r="A17" s="1" t="s">
         <v>65</v>
       </c>
@@ -1457,7 +1463,7 @@
       </c>
       <c r="H17" s="19"/>
     </row>
-    <row r="18" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" ht="16">
       <c r="A18" s="1" t="s">
         <v>65</v>
       </c>
@@ -1492,22 +1498,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J13"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="6.5" style="10" customWidth="1"/>
-    <col min="2" max="2" width="5.625" style="10" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.125" style="10" customWidth="1"/>
-    <col min="4" max="4" width="32.375" style="10" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.625" style="10" customWidth="1"/>
-    <col min="6" max="6" width="14.875" style="10" customWidth="1"/>
-    <col min="7" max="7" width="13.125" style="10" customWidth="1"/>
-    <col min="8" max="8" width="11.625" style="10" customWidth="1"/>
-    <col min="9" max="9" width="90.875" style="10" customWidth="1"/>
-    <col min="10" max="10" width="24.375" style="10" customWidth="1"/>
+    <col min="2" max="2" width="5.6640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.1640625" style="10" customWidth="1"/>
+    <col min="4" max="4" width="32.33203125" style="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.6640625" style="10" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" style="10" customWidth="1"/>
+    <col min="7" max="7" width="13.1640625" style="10" customWidth="1"/>
+    <col min="8" max="8" width="11.6640625" style="10" customWidth="1"/>
+    <col min="9" max="9" width="90.83203125" style="10" customWidth="1"/>
+    <col min="10" max="10" width="24.33203125" style="10" customWidth="1"/>
     <col min="11" max="16384" width="9" style="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1539,7 +1545,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
@@ -1571,7 +1577,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10">
       <c r="A3" s="1" t="s">
         <v>15</v>
       </c>
@@ -1589,7 +1595,7 @@
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10">
       <c r="A4" s="1" t="s">
         <v>17</v>
       </c>
@@ -1621,7 +1627,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="33" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" ht="34">
       <c r="A5" s="1" t="s">
         <v>18</v>
       </c>
@@ -1653,7 +1659,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10">
       <c r="A6" s="4">
         <v>10101</v>
       </c>
@@ -1685,7 +1691,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10">
       <c r="A7" s="4">
         <v>10102</v>
       </c>
@@ -1717,7 +1723,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10">
       <c r="A8" s="4">
         <v>10103</v>
       </c>
@@ -1749,7 +1755,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10">
       <c r="A9" s="4">
         <v>10104</v>
       </c>
@@ -1781,7 +1787,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10">
       <c r="A10" s="4">
         <v>10105</v>
       </c>
@@ -1813,7 +1819,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10">
       <c r="A11" s="4">
         <v>10201</v>
       </c>
@@ -1843,7 +1849,7 @@
       </c>
       <c r="J11" s="6"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10">
       <c r="A12" s="4">
         <v>10202</v>
       </c>
@@ -1873,7 +1879,7 @@
       </c>
       <c r="J12" s="6"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10">
       <c r="A13" s="4">
         <v>10203</v>
       </c>
@@ -1917,13 +1923,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06B4D15F-7CDD-ED40-889B-A4868E886B80}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="14.875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.125" style="16" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.1640625" style="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" ht="16">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1934,7 +1940,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" ht="16">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
@@ -1945,14 +1951,14 @@
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" ht="16">
       <c r="A3" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="22"/>
     </row>
-    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" ht="16">
       <c r="A4" s="1" t="s">
         <v>17</v>
       </c>
@@ -1963,7 +1969,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" ht="17">
       <c r="A5" s="1" t="s">
         <v>18</v>
       </c>
@@ -1972,7 +1978,7 @@
       </c>
       <c r="C5" s="22"/>
     </row>
-    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" ht="16">
       <c r="A6" s="4">
         <v>1</v>
       </c>
@@ -1983,7 +1989,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" ht="16">
       <c r="A7" s="4">
         <v>2</v>
       </c>
@@ -1994,7 +2000,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" ht="16">
       <c r="A8" s="4">
         <v>3</v>
       </c>
@@ -2005,7 +2011,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" ht="16">
       <c r="A9" s="4">
         <v>4</v>
       </c>
@@ -2016,14 +2022,14 @@
         <v>96</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" ht="16">
       <c r="A10" s="4">
         <v>5</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="21"/>
     </row>
-    <row r="11" spans="1:3" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" ht="16">
       <c r="A11" s="4">
         <v>6</v>
       </c>
@@ -2034,7 +2040,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" ht="16">
       <c r="A12" s="4">
         <v>7</v>
       </c>
@@ -2045,7 +2051,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" ht="16">
       <c r="A13" s="4">
         <v>8</v>
       </c>
@@ -2068,21 +2074,21 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E27B46D-4699-4B1C-B2B1-8A327D06725E}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.5" customWidth="1"/>
     <col min="2" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="11.625" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" s="27" customFormat="1">
       <c r="A1" s="28" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
-        <v>0</v>
+    <row r="2" spans="1:5" ht="16">
+      <c r="A2" s="7" t="s">
+        <v>118</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>1</v>
@@ -2097,7 +2103,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" ht="16">
       <c r="A3" s="1" t="s">
         <v>103</v>
       </c>
@@ -2114,7 +2120,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" ht="16">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
@@ -2125,7 +2131,7 @@
       <c r="D4" s="1"/>
       <c r="E4" s="2"/>
     </row>
-    <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" ht="16">
       <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
@@ -2142,7 +2148,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" ht="16">
       <c r="A6" s="1" t="s">
         <v>18</v>
       </c>
@@ -2155,7 +2161,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" ht="16">
       <c r="A7" s="25" t="s">
         <v>104</v>
       </c>
@@ -2172,7 +2178,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" ht="16">
       <c r="A8" s="25" t="s">
         <v>104</v>
       </c>
@@ -2189,7 +2195,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" ht="16">
       <c r="A9" s="25" t="s">
         <v>104</v>
       </c>
@@ -2206,7 +2212,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" ht="16">
       <c r="A10" s="25" t="s">
         <v>104</v>
       </c>
@@ -2235,19 +2241,19 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E541871-473E-3747-A4FF-7005DDAE5E45}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.5" customWidth="1"/>
     <col min="2" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="11.625" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" s="27" customFormat="1">
       <c r="A1" s="28" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" ht="16">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -2264,7 +2270,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" ht="16">
       <c r="A3" s="1" t="s">
         <v>103</v>
       </c>
@@ -2281,7 +2287,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" ht="16">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
@@ -2292,7 +2298,7 @@
       <c r="D4" s="1"/>
       <c r="E4" s="2"/>
     </row>
-    <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" ht="16">
       <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
@@ -2309,7 +2315,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" ht="16">
       <c r="A6" s="1" t="s">
         <v>18</v>
       </c>
@@ -2322,7 +2328,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" ht="16">
       <c r="A7" s="25" t="s">
         <v>104</v>
       </c>
@@ -2339,7 +2345,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" ht="16">
       <c r="A8" s="25" t="s">
         <v>104</v>
       </c>
@@ -2356,7 +2362,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" ht="16">
       <c r="A9" s="25" t="s">
         <v>104</v>
       </c>
@@ -2373,7 +2379,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" ht="16">
       <c r="A10" s="25" t="s">
         <v>104</v>
       </c>
@@ -2402,19 +2408,19 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D10B9FB-C914-9E4D-9ED5-4AA283A47ADC}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.5" customWidth="1"/>
     <col min="2" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="11.625" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" s="27" customFormat="1">
       <c r="A1" s="28" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" ht="16">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -2431,7 +2437,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" ht="16">
       <c r="A3" s="1" t="s">
         <v>103</v>
       </c>
@@ -2448,7 +2454,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" ht="16">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
@@ -2459,7 +2465,7 @@
       <c r="D4" s="1"/>
       <c r="E4" s="2"/>
     </row>
-    <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" ht="16">
       <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
@@ -2476,7 +2482,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" ht="16">
       <c r="A6" s="1" t="s">
         <v>18</v>
       </c>
@@ -2489,7 +2495,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" ht="16">
       <c r="A7" s="25" t="s">
         <v>104</v>
       </c>
@@ -2506,7 +2512,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" ht="16">
       <c r="A8" s="25" t="s">
         <v>104</v>
       </c>
@@ -2523,7 +2529,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" ht="16">
       <c r="A9" s="25" t="s">
         <v>104</v>
       </c>
@@ -2540,7 +2546,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" ht="16">
       <c r="A10" s="25" t="s">
         <v>104</v>
       </c>
@@ -2569,19 +2575,19 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CA9512F-15D7-C04B-B65B-D43362DB2865}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.5" customWidth="1"/>
     <col min="2" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="11.625" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" s="27" customFormat="1">
       <c r="A1" s="28" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" ht="16">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -2598,7 +2604,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" ht="16">
       <c r="A3" s="1" t="s">
         <v>103</v>
       </c>
@@ -2615,7 +2621,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" ht="16">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
@@ -2626,7 +2632,7 @@
       <c r="D4" s="1"/>
       <c r="E4" s="2"/>
     </row>
-    <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" ht="16">
       <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
@@ -2643,7 +2649,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" ht="16">
       <c r="A6" s="1" t="s">
         <v>18</v>
       </c>
@@ -2656,7 +2662,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" ht="16">
       <c r="A7" s="25" t="s">
         <v>104</v>
       </c>
@@ -2673,7 +2679,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" ht="16">
       <c r="A8" s="25" t="s">
         <v>104</v>
       </c>
@@ -2690,7 +2696,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" ht="16">
       <c r="A9" s="25" t="s">
         <v>104</v>
       </c>
@@ -2707,7 +2713,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" ht="16">
       <c r="A10" s="25" t="s">
         <v>104</v>
       </c>
@@ -2736,9 +2742,9 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADBB972E-C927-480C-A467-3665FD9F033A}">
   <dimension ref="B2"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:2">
       <c r="B2" s="24" t="s">
         <v>98</v>
       </c>

</xml_diff>